<commit_message>
Regenerate example outputs and restamp test outputs for v3.2022.3
- inst/testdata/examples_of_output: the 6 xlsx, 6 html and 3 pdf examples
  are regenerated, so report footers read "by EJAM v3.2022.3, 10/1/26,
  ACS 2018-2022" instead of v3.2022.2, 8/1/26.
- The 9 testoutput_* datasets were recomputed with the same calls as
  data-raw/. Every value is identical to the committed versions (0 differing
  elements); only their metadata changes (ejam_package_version and
  ejscreen_version 3.2022.3, ejscreen_releasedate 2026-10-01).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
+++ b/inst/testdata/examples_of_output/testoutput_ejam2excel_10pts_1miles.xlsx
@@ -5482,6 +5482,41 @@
     </dxf>
   </dxfs>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:oneCellAnchor xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+    <xdr:from xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+      <xdr:col xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">0</xdr:col>
+      <xdr:colOff xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">0</xdr:colOff>
+      <xdr:row xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">0</xdr:row>
+      <xdr:rowOff xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">0</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" cx="9144000" cy="45720000"/>
+    <xdr:pic xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+      <xdr:nvPicPr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+        <xdr:cNvPr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" id="1" name="Picture 1"/>
+        <xdr:cNvPicPr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+          <a:picLocks xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
+        </a:blip>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect">
+          <a:avLst xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
@@ -40063,6 +40098,7 @@
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId2"/>
+  <drawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>